<commit_message>
feat: add 3rd tier treatment to clinical_data.xlsx
</commit_message>
<xml_diff>
--- a/data/input/clinical_data/clinical_data.xlsx
+++ b/data/input/clinical_data/clinical_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S86"/>
+  <dimension ref="A1:T86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -524,6 +524,11 @@
           <t>analysis_population</t>
         </is>
       </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>trait_niv_3_r</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -591,6 +596,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -658,6 +668,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -729,6 +744,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -802,6 +822,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -875,6 +900,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -946,6 +976,11 @@
       <c r="S7" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -1019,6 +1054,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1090,6 +1130,7 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1163,6 +1204,11 @@
       <c r="S10" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -1224,6 +1270,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1299,6 +1350,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1372,6 +1428,11 @@
       <c r="S13" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -1443,6 +1504,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1514,6 +1580,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1587,6 +1658,11 @@
       <c r="S16" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -1624,6 +1700,11 @@
           <t>ITT</t>
         </is>
       </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1691,6 +1772,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1758,6 +1844,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1827,6 +1918,11 @@
       <c r="S20" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -1898,6 +1994,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1969,6 +2070,11 @@
       <c r="S22" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -2040,6 +2146,11 @@
           <t>mITT</t>
         </is>
       </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2113,6 +2224,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2186,6 +2302,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2259,6 +2380,11 @@
       <c r="S26" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -2328,6 +2454,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2403,6 +2534,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2478,6 +2614,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2551,6 +2692,11 @@
       <c r="S30" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -2618,6 +2764,11 @@
       <c r="S31" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -2691,6 +2842,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2756,6 +2912,11 @@
       <c r="S33" t="inlineStr">
         <is>
           <t>ITT</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -2829,6 +2990,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2904,6 +3070,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2977,6 +3148,11 @@
       <c r="S36" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -3050,6 +3226,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3123,6 +3304,11 @@
       <c r="S38" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -3196,6 +3382,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3269,6 +3460,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3342,6 +3538,11 @@
       <c r="S41" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -3407,6 +3608,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3480,6 +3686,11 @@
       <c r="S43" t="inlineStr">
         <is>
           <t>mITT</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -3547,6 +3758,11 @@
       <c r="S44" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -3620,6 +3836,11 @@
           <t>mITT</t>
         </is>
       </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3691,6 +3912,7 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3758,6 +3980,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3831,6 +4058,11 @@
       <c r="S48" t="inlineStr">
         <is>
           <t>ITT</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -3902,6 +4134,11 @@
       <c r="S49" t="inlineStr">
         <is>
           <t>mITT</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -3973,6 +4210,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4046,6 +4288,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4113,6 +4360,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4178,6 +4430,11 @@
       <c r="S53" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -4221,6 +4478,11 @@
           <t>Aucune Analyse</t>
         </is>
       </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4296,6 +4558,7 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4371,6 +4634,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4444,6 +4712,11 @@
       <c r="S57" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -4513,6 +4786,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4586,6 +4864,11 @@
       <c r="S59" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -4655,6 +4938,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4730,6 +5018,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4803,6 +5096,11 @@
       <c r="S62" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -4872,6 +5170,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4945,6 +5248,11 @@
       <c r="S64" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -5014,6 +5322,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5089,6 +5402,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5162,6 +5480,11 @@
       <c r="S67" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -5227,6 +5550,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5300,6 +5628,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5375,6 +5708,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5450,6 +5788,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5525,6 +5868,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5598,6 +5946,11 @@
       <c r="S73" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -5667,6 +6020,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5740,6 +6098,11 @@
       <c r="S75" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -5813,6 +6176,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5878,6 +6246,11 @@
       <c r="S77" t="inlineStr">
         <is>
           <t>mITT</t>
+        </is>
+      </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -5943,6 +6316,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6010,6 +6388,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6083,6 +6466,11 @@
       <c r="S80" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -6156,6 +6544,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6223,6 +6616,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6296,6 +6694,11 @@
       <c r="S83" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -6369,6 +6772,11 @@
       <c r="S84" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -6440,6 +6848,11 @@
       <c r="S85" t="inlineStr">
         <is>
           <t>PP</t>
+        </is>
+      </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -6511,6 +6924,11 @@
           <t>PP</t>
         </is>
       </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: add pupillary reactivity to clinical data
</commit_message>
<xml_diff>
--- a/data/input/clinical_data/clinical_data.xlsx
+++ b/data/input/clinical_data/clinical_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T86"/>
+  <dimension ref="A1:U86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,6 +529,11 @@
           <t>trait_niv_3_r</t>
         </is>
       </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>bl_reac_pupill_r</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -601,6 +606,7 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -673,6 +679,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -749,6 +760,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -827,6 +843,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -905,6 +926,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -981,6 +1007,11 @@
       <c r="T7" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1059,6 +1090,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1131,6 +1167,7 @@
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1209,6 +1246,11 @@
       <c r="T10" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1275,6 +1317,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1355,6 +1402,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1433,6 +1485,11 @@
       <c r="T13" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1509,6 +1566,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1585,6 +1647,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1663,6 +1730,11 @@
       <c r="T16" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1705,6 +1777,7 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1777,6 +1850,7 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1849,6 +1923,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1923,6 +2002,11 @@
       <c r="T20" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1999,6 +2083,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2075,6 +2164,11 @@
       <c r="T22" t="inlineStr">
         <is>
           <t>Oui</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -2151,6 +2245,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2229,6 +2328,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2307,6 +2411,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2385,6 +2494,11 @@
       <c r="T26" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -2459,6 +2573,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2539,6 +2658,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2619,6 +2743,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2697,6 +2826,11 @@
       <c r="T30" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -2769,6 +2903,11 @@
       <c r="T31" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -2847,6 +2986,7 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2917,6 +3057,11 @@
       <c r="T33" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -2995,6 +3140,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3075,6 +3225,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3153,6 +3308,11 @@
       <c r="T36" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -3231,6 +3391,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3309,6 +3474,11 @@
       <c r="T38" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -3387,6 +3557,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3465,6 +3640,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3543,6 +3723,11 @@
       <c r="T41" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -3613,6 +3798,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3691,6 +3881,11 @@
       <c r="T43" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -3763,6 +3958,11 @@
       <c r="T44" t="inlineStr">
         <is>
           <t>Oui</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -3841,6 +4041,7 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3913,6 +4114,11 @@
         </is>
       </c>
       <c r="T46" t="inlineStr"/>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3985,6 +4191,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4063,6 +4274,11 @@
       <c r="T48" t="inlineStr">
         <is>
           <t>Oui</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -4139,6 +4355,11 @@
       <c r="T49" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -4215,6 +4436,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4293,6 +4519,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4365,6 +4596,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4435,6 +4671,11 @@
       <c r="T53" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -4483,6 +4724,7 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4559,6 +4801,11 @@
         </is>
       </c>
       <c r="T55" t="inlineStr"/>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4639,6 +4886,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4717,6 +4969,11 @@
       <c r="T57" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -4791,6 +5048,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4869,6 +5131,11 @@
       <c r="T59" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -4943,6 +5210,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5023,6 +5295,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5101,6 +5378,11 @@
       <c r="T62" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -5175,6 +5457,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5253,6 +5540,11 @@
       <c r="T64" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -5327,6 +5619,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5407,6 +5704,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5485,6 +5787,11 @@
       <c r="T67" t="inlineStr">
         <is>
           <t>Oui</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -5555,6 +5862,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5633,6 +5945,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5713,6 +6030,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5793,6 +6115,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5873,6 +6200,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5951,6 +6283,11 @@
       <c r="T73" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -6025,6 +6362,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6103,6 +6445,11 @@
       <c r="T75" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -6181,6 +6528,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6251,6 +6603,11 @@
       <c r="T77" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -6321,6 +6678,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6393,6 +6755,11 @@
           <t>Oui</t>
         </is>
       </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6471,6 +6838,11 @@
       <c r="T80" t="inlineStr">
         <is>
           <t>Oui</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -6549,6 +6921,7 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6621,6 +6994,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6699,6 +7077,11 @@
       <c r="T83" t="inlineStr">
         <is>
           <t>Oui</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -6777,6 +7160,11 @@
       <c r="T84" t="inlineStr">
         <is>
           <t>Oui</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -6855,6 +7243,7 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6929,6 +7318,11 @@
           <t>Non</t>
         </is>
       </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: add cumulative time of dose ICP
</commit_message>
<xml_diff>
--- a/data/input/clinical_data/clinical_data.xlsx
+++ b/data/input/clinical_data/clinical_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U86"/>
+  <dimension ref="A1:V86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,6 +534,11 @@
           <t>bl_reac_pupill_r</t>
         </is>
       </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>dose_PIC_temps_prct</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -607,6 +612,11 @@
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -679,9 +689,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U3" t="n">
+        <v>2</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>23</t>
         </is>
       </c>
     </row>
@@ -760,9 +773,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U4" t="n">
+        <v>2</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -843,7 +859,10 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="U5" t="n">
+        <v>2</v>
+      </c>
+      <c r="V5" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -926,9 +945,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U6" t="n">
+        <v>2</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -1009,9 +1031,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U7" t="n">
+        <v>2</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1090,9 +1115,12 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U8" t="n">
+        <v>2</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -1168,6 +1196,7 @@
       </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1248,9 +1277,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U10" t="n">
+        <v>2</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -1317,9 +1349,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U11" t="n">
+        <v>2</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1402,9 +1437,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="U12" t="n">
+        <v>1</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -1487,9 +1525,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U13" t="n">
+        <v>2</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -1566,9 +1607,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U14" t="n">
+        <v>2</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>51</t>
         </is>
       </c>
     </row>
@@ -1647,9 +1691,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U15" t="n">
+        <v>2</v>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -1732,9 +1779,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U16" t="n">
+        <v>2</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1778,6 +1828,11 @@
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1851,6 +1906,11 @@
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1923,9 +1983,12 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U19" t="n">
+        <v>2</v>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -2004,9 +2067,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U20" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -2083,9 +2149,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U21" t="n">
+        <v>2</v>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>38</t>
         </is>
       </c>
     </row>
@@ -2166,9 +2235,12 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -2245,7 +2317,10 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="U23" t="n">
+        <v>0</v>
+      </c>
+      <c r="V23" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -2328,9 +2403,12 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U24" t="n">
+        <v>2</v>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2489,10 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
+      <c r="U25" t="n">
+        <v>2</v>
+      </c>
+      <c r="V25" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -2496,9 +2577,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U26" t="n">
+        <v>2</v>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2573,9 +2657,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U27" t="n">
+        <v>2</v>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -2658,9 +2745,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U28" t="n">
+        <v>2</v>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -2743,9 +2833,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U29" t="n">
+        <v>2</v>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -2828,7 +2921,10 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr">
+      <c r="U30" t="n">
+        <v>0</v>
+      </c>
+      <c r="V30" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -2905,9 +3001,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U31" t="n">
+        <v>2</v>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2987,6 +3086,11 @@
         </is>
       </c>
       <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3059,9 +3163,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U33" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U33" t="n">
+        <v>2</v>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -3140,9 +3247,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U34" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U34" t="n">
+        <v>2</v>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -3225,9 +3335,12 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U35" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="U35" t="n">
+        <v>1</v>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>16</t>
         </is>
       </c>
     </row>
@@ -3310,9 +3423,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U36" t="n">
+        <v>2</v>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -3391,9 +3507,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U37" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U37" t="n">
+        <v>2</v>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -3476,9 +3595,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U38" t="n">
+        <v>0</v>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -3557,9 +3679,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U39" t="n">
+        <v>0</v>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -3640,9 +3765,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U40" t="n">
+        <v>0</v>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -3725,9 +3853,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U41" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U41" t="n">
+        <v>2</v>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -3798,9 +3929,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U42" t="n">
+        <v>0</v>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -3883,9 +4017,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U43" t="n">
+        <v>2</v>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -3960,9 +4097,12 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U44" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U44" t="n">
+        <v>0</v>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -4042,6 +4182,11 @@
         </is>
       </c>
       <c r="U45" t="inlineStr"/>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4114,9 +4259,12 @@
         </is>
       </c>
       <c r="T46" t="inlineStr"/>
-      <c r="U46" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U46" t="n">
+        <v>2</v>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -4191,9 +4339,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U47" t="n">
+        <v>2</v>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -4276,9 +4427,12 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U48" t="n">
+        <v>0</v>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -4357,9 +4511,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U49" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="U49" t="n">
+        <v>1</v>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -4436,9 +4593,12 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U50" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U50" t="n">
+        <v>0</v>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -4519,9 +4679,12 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U51" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U51" t="n">
+        <v>2</v>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -4596,9 +4759,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U52" t="n">
+        <v>2</v>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -4673,9 +4839,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U53" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U53" t="n">
+        <v>2</v>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -4725,6 +4894,11 @@
         </is>
       </c>
       <c r="U54" t="inlineStr"/>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4801,11 +4975,10 @@
         </is>
       </c>
       <c r="T55" t="inlineStr"/>
-      <c r="U55" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="U55" t="n">
+        <v>2</v>
+      </c>
+      <c r="V55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4886,9 +5059,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U56" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U56" t="n">
+        <v>2</v>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -4971,9 +5147,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U57" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U57" t="n">
+        <v>2</v>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -5048,9 +5227,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U58" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U58" t="n">
+        <v>2</v>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -5133,9 +5315,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U59" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U59" t="n">
+        <v>2</v>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -5210,9 +5395,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U60" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U60" t="n">
+        <v>0</v>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -5295,9 +5483,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U61" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U61" t="n">
+        <v>0</v>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -5380,9 +5571,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U62" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U62" t="n">
+        <v>2</v>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -5457,9 +5651,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U63" t="n">
+        <v>2</v>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -5542,9 +5739,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U64" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U64" t="n">
+        <v>2</v>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -5619,7 +5819,10 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U65" t="inlineStr">
+      <c r="U65" t="n">
+        <v>2</v>
+      </c>
+      <c r="V65" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -5704,9 +5907,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U66" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U66" t="n">
+        <v>2</v>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -5789,9 +5995,12 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U67" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U67" t="n">
+        <v>2</v>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -5862,9 +6071,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U68" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U68" t="n">
+        <v>2</v>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -5945,9 +6157,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U69" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U69" t="n">
+        <v>0</v>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -6030,9 +6245,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U70" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U70" t="n">
+        <v>2</v>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -6115,9 +6333,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U71" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U71" t="n">
+        <v>0</v>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -6200,9 +6421,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U72" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U72" t="n">
+        <v>2</v>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -6285,9 +6509,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U73" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U73" t="n">
+        <v>0</v>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -6362,9 +6589,12 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U74" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U74" t="n">
+        <v>0</v>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6677,10 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U75" t="inlineStr">
+      <c r="U75" t="n">
+        <v>2</v>
+      </c>
+      <c r="V75" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -6528,9 +6761,12 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U76" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U76" t="n">
+        <v>2</v>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>17</t>
         </is>
       </c>
     </row>
@@ -6605,9 +6841,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U77" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U77" t="n">
+        <v>2</v>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>24</t>
         </is>
       </c>
     </row>
@@ -6678,9 +6917,12 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U78" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U78" t="n">
+        <v>0</v>
+      </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -6755,7 +6997,10 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U79" t="inlineStr">
+      <c r="U79" t="n">
+        <v>0</v>
+      </c>
+      <c r="V79" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -6840,9 +7085,12 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U80" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U80" t="n">
+        <v>0</v>
+      </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -6922,6 +7170,11 @@
         </is>
       </c>
       <c r="U81" t="inlineStr"/>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6994,7 +7247,10 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U82" t="inlineStr">
+      <c r="U82" t="n">
+        <v>2</v>
+      </c>
+      <c r="V82" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -7079,9 +7335,12 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U83" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U83" t="n">
+        <v>2</v>
+      </c>
+      <c r="V83" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -7162,9 +7421,12 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="U84" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U84" t="n">
+        <v>2</v>
+      </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -7244,6 +7506,11 @@
         </is>
       </c>
       <c r="U85" t="inlineStr"/>
+      <c r="V85" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7318,9 +7585,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="U86" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="U86" t="n">
+        <v>0</v>
+      </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add initial_intracranial_pressure to clinical_data.xlsx
</commit_message>
<xml_diff>
--- a/data/input/clinical_data/clinical_data.xlsx
+++ b/data/input/clinical_data/clinical_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V86"/>
+  <dimension ref="A1:W86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,6 +539,11 @@
           <t>dose_PIC_temps_prct</t>
         </is>
       </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>PIC_H0</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -612,9 +617,12 @@
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>7</t>
+      <c r="V2" t="n">
+        <v>7</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -692,9 +700,12 @@
       <c r="U3" t="n">
         <v>2</v>
       </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>23</t>
+      <c r="V3" t="n">
+        <v>23</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -776,9 +787,12 @@
       <c r="U4" t="n">
         <v>2</v>
       </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>11</t>
+      <c r="V4" t="n">
+        <v>11</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -862,9 +876,12 @@
       <c r="U5" t="n">
         <v>2</v>
       </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="V5" t="n">
+        <v>2</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -948,9 +965,12 @@
       <c r="U6" t="n">
         <v>2</v>
       </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>8</t>
+      <c r="V6" t="n">
+        <v>8</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -1034,9 +1054,12 @@
       <c r="U7" t="n">
         <v>2</v>
       </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="V7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -1118,9 +1141,12 @@
       <c r="U8" t="n">
         <v>2</v>
       </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="V8" t="n">
+        <v>3</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>23</t>
         </is>
       </c>
     </row>
@@ -1197,6 +1223,11 @@
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1280,9 +1311,12 @@
       <c r="U10" t="n">
         <v>2</v>
       </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>8</t>
+      <c r="V10" t="n">
+        <v>8</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -1352,9 +1386,12 @@
       <c r="U11" t="n">
         <v>2</v>
       </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>4</t>
+      <c r="V11" t="n">
+        <v>4</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -1440,9 +1477,12 @@
       <c r="U12" t="n">
         <v>1</v>
       </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="V12" t="n">
+        <v>3</v>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>14</t>
         </is>
       </c>
     </row>
@@ -1528,9 +1568,12 @@
       <c r="U13" t="n">
         <v>2</v>
       </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="V13" t="n">
+        <v>3</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>19</t>
         </is>
       </c>
     </row>
@@ -1610,9 +1653,12 @@
       <c r="U14" t="n">
         <v>2</v>
       </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>51</t>
+      <c r="V14" t="n">
+        <v>51</v>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -1694,9 +1740,12 @@
       <c r="U15" t="n">
         <v>2</v>
       </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="V15" t="n">
+        <v>3</v>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -1782,9 +1831,12 @@
       <c r="U16" t="n">
         <v>2</v>
       </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>4</t>
+      <c r="V16" t="n">
+        <v>4</v>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>14</t>
         </is>
       </c>
     </row>
@@ -1828,11 +1880,10 @@
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="V17" t="n">
+        <v>3</v>
+      </c>
+      <c r="W17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1906,9 +1957,12 @@
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>11</t>
+      <c r="V18" t="n">
+        <v>11</v>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1986,9 +2040,12 @@
       <c r="U19" t="n">
         <v>2</v>
       </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>10</t>
+      <c r="V19" t="n">
+        <v>10</v>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>30</t>
         </is>
       </c>
     </row>
@@ -2070,9 +2127,12 @@
       <c r="U20" t="n">
         <v>0</v>
       </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="V20" t="n">
+        <v>2</v>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>17</t>
         </is>
       </c>
     </row>
@@ -2152,9 +2212,12 @@
       <c r="U21" t="n">
         <v>2</v>
       </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>38</t>
+      <c r="V21" t="n">
+        <v>38</v>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -2238,9 +2301,12 @@
       <c r="U22" t="n">
         <v>0</v>
       </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>11</t>
+      <c r="V22" t="n">
+        <v>11</v>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2386,10 @@
       <c r="U23" t="n">
         <v>0</v>
       </c>
-      <c r="V23" t="inlineStr">
+      <c r="V23" t="n">
+        <v>0</v>
+      </c>
+      <c r="W23" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -2406,9 +2475,12 @@
       <c r="U24" t="n">
         <v>2</v>
       </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>4</t>
+      <c r="V24" t="n">
+        <v>4</v>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -2492,9 +2564,12 @@
       <c r="U25" t="n">
         <v>2</v>
       </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="V25" t="n">
+        <v>2</v>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>16</t>
         </is>
       </c>
     </row>
@@ -2580,11 +2655,10 @@
       <c r="U26" t="n">
         <v>2</v>
       </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="V26" t="n">
+        <v>1</v>
+      </c>
+      <c r="W26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2660,9 +2734,12 @@
       <c r="U27" t="n">
         <v>2</v>
       </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="V27" t="n">
+        <v>0</v>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2748,11 +2825,10 @@
       <c r="U28" t="n">
         <v>2</v>
       </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="V28" t="n">
+        <v>0</v>
+      </c>
+      <c r="W28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2836,9 +2912,12 @@
       <c r="U29" t="n">
         <v>2</v>
       </c>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="V29" t="n">
+        <v>0</v>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -2924,9 +3003,12 @@
       <c r="U30" t="n">
         <v>0</v>
       </c>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="V30" t="n">
+        <v>0</v>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -3004,9 +3086,12 @@
       <c r="U31" t="n">
         <v>2</v>
       </c>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="V31" t="n">
+        <v>3</v>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -3086,9 +3171,12 @@
         </is>
       </c>
       <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="V32" t="n">
+        <v>0</v>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -3166,9 +3254,12 @@
       <c r="U33" t="n">
         <v>2</v>
       </c>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="V33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -3250,9 +3341,12 @@
       <c r="U34" t="n">
         <v>2</v>
       </c>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="V34" t="n">
+        <v>3</v>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -3338,9 +3432,12 @@
       <c r="U35" t="n">
         <v>1</v>
       </c>
-      <c r="V35" t="inlineStr">
-        <is>
-          <t>16</t>
+      <c r="V35" t="n">
+        <v>16</v>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>25</t>
         </is>
       </c>
     </row>
@@ -3426,9 +3523,12 @@
       <c r="U36" t="n">
         <v>2</v>
       </c>
-      <c r="V36" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="V36" t="n">
+        <v>3</v>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -3510,7 +3610,10 @@
       <c r="U37" t="n">
         <v>2</v>
       </c>
-      <c r="V37" t="inlineStr">
+      <c r="V37" t="n">
+        <v>0</v>
+      </c>
+      <c r="W37" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -3598,9 +3701,12 @@
       <c r="U38" t="n">
         <v>0</v>
       </c>
-      <c r="V38" t="inlineStr">
-        <is>
-          <t>6</t>
+      <c r="V38" t="n">
+        <v>6</v>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -3682,9 +3788,12 @@
       <c r="U39" t="n">
         <v>0</v>
       </c>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>11</t>
+      <c r="V39" t="n">
+        <v>11</v>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -3768,9 +3877,12 @@
       <c r="U40" t="n">
         <v>0</v>
       </c>
-      <c r="V40" t="inlineStr">
-        <is>
-          <t>7</t>
+      <c r="V40" t="n">
+        <v>7</v>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -3856,9 +3968,12 @@
       <c r="U41" t="n">
         <v>2</v>
       </c>
-      <c r="V41" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="V41" t="n">
+        <v>0</v>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>19</t>
         </is>
       </c>
     </row>
@@ -3932,9 +4047,12 @@
       <c r="U42" t="n">
         <v>0</v>
       </c>
-      <c r="V42" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="V42" t="n">
+        <v>1</v>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -4020,9 +4138,12 @@
       <c r="U43" t="n">
         <v>2</v>
       </c>
-      <c r="V43" t="inlineStr">
-        <is>
-          <t>4</t>
+      <c r="V43" t="n">
+        <v>4</v>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -4100,9 +4221,12 @@
       <c r="U44" t="n">
         <v>0</v>
       </c>
-      <c r="V44" t="inlineStr">
-        <is>
-          <t>6</t>
+      <c r="V44" t="n">
+        <v>6</v>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -4182,9 +4306,12 @@
         </is>
       </c>
       <c r="U45" t="inlineStr"/>
-      <c r="V45" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="V45" t="n">
+        <v>2</v>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>19</t>
         </is>
       </c>
     </row>
@@ -4262,9 +4389,12 @@
       <c r="U46" t="n">
         <v>2</v>
       </c>
-      <c r="V46" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="V46" t="n">
+        <v>0</v>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -4342,9 +4472,12 @@
       <c r="U47" t="n">
         <v>2</v>
       </c>
-      <c r="V47" t="inlineStr">
-        <is>
-          <t>8</t>
+      <c r="V47" t="n">
+        <v>8</v>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>24</t>
         </is>
       </c>
     </row>
@@ -4430,9 +4563,12 @@
       <c r="U48" t="n">
         <v>0</v>
       </c>
-      <c r="V48" t="inlineStr">
-        <is>
-          <t>18</t>
+      <c r="V48" t="n">
+        <v>18</v>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -4514,9 +4650,12 @@
       <c r="U49" t="n">
         <v>1</v>
       </c>
-      <c r="V49" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="V49" t="n">
+        <v>0</v>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>13</t>
         </is>
       </c>
     </row>
@@ -4596,9 +4735,12 @@
       <c r="U50" t="n">
         <v>0</v>
       </c>
-      <c r="V50" t="inlineStr">
-        <is>
-          <t>8</t>
+      <c r="V50" t="n">
+        <v>8</v>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -4682,9 +4824,12 @@
       <c r="U51" t="n">
         <v>2</v>
       </c>
-      <c r="V51" t="inlineStr">
-        <is>
-          <t>12</t>
+      <c r="V51" t="n">
+        <v>12</v>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -4762,9 +4907,12 @@
       <c r="U52" t="n">
         <v>2</v>
       </c>
-      <c r="V52" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="V52" t="n">
+        <v>0</v>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -4842,9 +4990,12 @@
       <c r="U53" t="n">
         <v>2</v>
       </c>
-      <c r="V53" t="inlineStr">
-        <is>
-          <t>6</t>
+      <c r="V53" t="n">
+        <v>6</v>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -4894,11 +5045,10 @@
         </is>
       </c>
       <c r="U54" t="inlineStr"/>
-      <c r="V54" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="V54" t="n">
+        <v>0</v>
+      </c>
+      <c r="W54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4979,6 +5129,11 @@
         <v>2</v>
       </c>
       <c r="V55" t="inlineStr"/>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5062,9 +5217,12 @@
       <c r="U56" t="n">
         <v>2</v>
       </c>
-      <c r="V56" t="inlineStr">
-        <is>
-          <t>4</t>
+      <c r="V56" t="n">
+        <v>4</v>
+      </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -5150,11 +5308,10 @@
       <c r="U57" t="n">
         <v>2</v>
       </c>
-      <c r="V57" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="V57" t="n">
+        <v>3</v>
+      </c>
+      <c r="W57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5230,9 +5387,12 @@
       <c r="U58" t="n">
         <v>2</v>
       </c>
-      <c r="V58" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="V58" t="n">
+        <v>1</v>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -5318,11 +5478,10 @@
       <c r="U59" t="n">
         <v>2</v>
       </c>
-      <c r="V59" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="V59" t="n">
+        <v>3</v>
+      </c>
+      <c r="W59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5398,11 +5557,10 @@
       <c r="U60" t="n">
         <v>0</v>
       </c>
-      <c r="V60" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="V60" t="n">
+        <v>1</v>
+      </c>
+      <c r="W60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5486,9 +5644,12 @@
       <c r="U61" t="n">
         <v>0</v>
       </c>
-      <c r="V61" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="V61" t="n">
+        <v>3</v>
+      </c>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -5574,9 +5735,12 @@
       <c r="U62" t="n">
         <v>2</v>
       </c>
-      <c r="V62" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="V62" t="n">
+        <v>1</v>
+      </c>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -5654,9 +5818,12 @@
       <c r="U63" t="n">
         <v>2</v>
       </c>
-      <c r="V63" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="V63" t="n">
+        <v>3</v>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -5742,9 +5909,12 @@
       <c r="U64" t="n">
         <v>2</v>
       </c>
-      <c r="V64" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="V64" t="n">
+        <v>3</v>
+      </c>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -5822,9 +5992,12 @@
       <c r="U65" t="n">
         <v>2</v>
       </c>
-      <c r="V65" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="V65" t="n">
+        <v>2</v>
+      </c>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -5910,9 +6083,12 @@
       <c r="U66" t="n">
         <v>2</v>
       </c>
-      <c r="V66" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="V66" t="n">
+        <v>0</v>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>34</t>
         </is>
       </c>
     </row>
@@ -5998,9 +6174,12 @@
       <c r="U67" t="n">
         <v>2</v>
       </c>
-      <c r="V67" t="inlineStr">
-        <is>
-          <t>11</t>
+      <c r="V67" t="n">
+        <v>11</v>
+      </c>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -6074,9 +6253,12 @@
       <c r="U68" t="n">
         <v>2</v>
       </c>
-      <c r="V68" t="inlineStr">
-        <is>
-          <t>9</t>
+      <c r="V68" t="n">
+        <v>9</v>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>17</t>
         </is>
       </c>
     </row>
@@ -6160,9 +6342,12 @@
       <c r="U69" t="n">
         <v>0</v>
       </c>
-      <c r="V69" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="V69" t="n">
+        <v>3</v>
+      </c>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t>17</t>
         </is>
       </c>
     </row>
@@ -6248,7 +6433,10 @@
       <c r="U70" t="n">
         <v>2</v>
       </c>
-      <c r="V70" t="inlineStr">
+      <c r="V70" t="n">
+        <v>0</v>
+      </c>
+      <c r="W70" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -6336,11 +6524,10 @@
       <c r="U71" t="n">
         <v>0</v>
       </c>
-      <c r="V71" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="V71" t="n">
+        <v>3</v>
+      </c>
+      <c r="W71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6424,9 +6611,12 @@
       <c r="U72" t="n">
         <v>2</v>
       </c>
-      <c r="V72" t="inlineStr">
-        <is>
-          <t>10</t>
+      <c r="V72" t="n">
+        <v>10</v>
+      </c>
+      <c r="W72" t="inlineStr">
+        <is>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -6512,9 +6702,12 @@
       <c r="U73" t="n">
         <v>0</v>
       </c>
-      <c r="V73" t="inlineStr">
-        <is>
-          <t>4</t>
+      <c r="V73" t="n">
+        <v>4</v>
+      </c>
+      <c r="W73" t="inlineStr">
+        <is>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -6592,9 +6785,12 @@
       <c r="U74" t="n">
         <v>0</v>
       </c>
-      <c r="V74" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="V74" t="n">
+        <v>3</v>
+      </c>
+      <c r="W74" t="inlineStr">
+        <is>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -6680,9 +6876,12 @@
       <c r="U75" t="n">
         <v>2</v>
       </c>
-      <c r="V75" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="V75" t="n">
+        <v>2</v>
+      </c>
+      <c r="W75" t="inlineStr">
+        <is>
+          <t>24</t>
         </is>
       </c>
     </row>
@@ -6764,9 +6963,12 @@
       <c r="U76" t="n">
         <v>2</v>
       </c>
-      <c r="V76" t="inlineStr">
-        <is>
-          <t>17</t>
+      <c r="V76" t="n">
+        <v>17</v>
+      </c>
+      <c r="W76" t="inlineStr">
+        <is>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -6844,9 +7046,12 @@
       <c r="U77" t="n">
         <v>2</v>
       </c>
-      <c r="V77" t="inlineStr">
-        <is>
-          <t>24</t>
+      <c r="V77" t="n">
+        <v>24</v>
+      </c>
+      <c r="W77" t="inlineStr">
+        <is>
+          <t>16</t>
         </is>
       </c>
     </row>
@@ -6920,11 +7125,10 @@
       <c r="U78" t="n">
         <v>0</v>
       </c>
-      <c r="V78" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="V78" t="n">
+        <v>3</v>
+      </c>
+      <c r="W78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7000,11 +7204,10 @@
       <c r="U79" t="n">
         <v>0</v>
       </c>
-      <c r="V79" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="V79" t="n">
+        <v>0</v>
+      </c>
+      <c r="W79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -7088,9 +7291,12 @@
       <c r="U80" t="n">
         <v>0</v>
       </c>
-      <c r="V80" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="V80" t="n">
+        <v>2</v>
+      </c>
+      <c r="W80" t="inlineStr">
+        <is>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -7170,11 +7376,10 @@
         </is>
       </c>
       <c r="U81" t="inlineStr"/>
-      <c r="V81" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="V81" t="n">
+        <v>2</v>
+      </c>
+      <c r="W81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7250,9 +7455,12 @@
       <c r="U82" t="n">
         <v>2</v>
       </c>
-      <c r="V82" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="V82" t="n">
+        <v>2</v>
+      </c>
+      <c r="W82" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -7338,9 +7546,12 @@
       <c r="U83" t="n">
         <v>2</v>
       </c>
-      <c r="V83" t="inlineStr">
-        <is>
-          <t>29</t>
+      <c r="V83" t="n">
+        <v>29</v>
+      </c>
+      <c r="W83" t="inlineStr">
+        <is>
+          <t>16</t>
         </is>
       </c>
     </row>
@@ -7424,11 +7635,10 @@
       <c r="U84" t="n">
         <v>2</v>
       </c>
-      <c r="V84" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+      <c r="V84" t="n">
+        <v>10</v>
+      </c>
+      <c r="W84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7506,11 +7716,10 @@
         </is>
       </c>
       <c r="U85" t="inlineStr"/>
-      <c r="V85" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="V85" t="n">
+        <v>0</v>
+      </c>
+      <c r="W85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7588,9 +7797,12 @@
       <c r="U86" t="n">
         <v>0</v>
       </c>
-      <c r="V86" t="inlineStr">
-        <is>
-          <t>5</t>
+      <c r="V86" t="n">
+        <v>5</v>
+      </c>
+      <c r="W86" t="inlineStr">
+        <is>
+          <t>9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add initial mean blood arterial pressure and cerebral perfusion pressure to clinical_data.xlsx
</commit_message>
<xml_diff>
--- a/data/input/clinical_data/clinical_data.xlsx
+++ b/data/input/clinical_data/clinical_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W86"/>
+  <dimension ref="A1:Y86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,6 +544,16 @@
           <t>PIC_H0</t>
         </is>
       </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>PAM_H0</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>PPC_H0</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -620,9 +630,15 @@
       <c r="V2" t="n">
         <v>7</v>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>10</t>
+      <c r="W2" t="n">
+        <v>10</v>
+      </c>
+      <c r="X2" t="n">
+        <v>87</v>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>77</t>
         </is>
       </c>
     </row>
@@ -703,9 +719,15 @@
       <c r="V3" t="n">
         <v>23</v>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>8</t>
+      <c r="W3" t="n">
+        <v>8</v>
+      </c>
+      <c r="X3" t="n">
+        <v>71</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>63</t>
         </is>
       </c>
     </row>
@@ -790,9 +812,15 @@
       <c r="V4" t="n">
         <v>11</v>
       </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>10</t>
+      <c r="W4" t="n">
+        <v>10</v>
+      </c>
+      <c r="X4" t="n">
+        <v>74</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>64</t>
         </is>
       </c>
     </row>
@@ -879,9 +907,15 @@
       <c r="V5" t="n">
         <v>2</v>
       </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>11</t>
+      <c r="W5" t="n">
+        <v>11</v>
+      </c>
+      <c r="X5" t="n">
+        <v>77</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>66</t>
         </is>
       </c>
     </row>
@@ -968,9 +1002,15 @@
       <c r="V6" t="n">
         <v>8</v>
       </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>11</t>
+      <c r="W6" t="n">
+        <v>11</v>
+      </c>
+      <c r="X6" t="n">
+        <v>79</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>68</t>
         </is>
       </c>
     </row>
@@ -1057,9 +1097,15 @@
       <c r="V7" t="n">
         <v>1</v>
       </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>8</t>
+      <c r="W7" t="n">
+        <v>8</v>
+      </c>
+      <c r="X7" t="n">
+        <v>79</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>71</t>
         </is>
       </c>
     </row>
@@ -1144,9 +1190,15 @@
       <c r="V8" t="n">
         <v>3</v>
       </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>23</t>
+      <c r="W8" t="n">
+        <v>23</v>
+      </c>
+      <c r="X8" t="n">
+        <v>90</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>67</t>
         </is>
       </c>
     </row>
@@ -1223,9 +1275,15 @@
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>5</t>
+      <c r="W9" t="n">
+        <v>5</v>
+      </c>
+      <c r="X9" t="n">
+        <v>86</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>81</t>
         </is>
       </c>
     </row>
@@ -1314,9 +1372,15 @@
       <c r="V10" t="n">
         <v>8</v>
       </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>10</t>
+      <c r="W10" t="n">
+        <v>10</v>
+      </c>
+      <c r="X10" t="n">
+        <v>84</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>74</t>
         </is>
       </c>
     </row>
@@ -1389,9 +1453,15 @@
       <c r="V11" t="n">
         <v>4</v>
       </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="W11" t="n">
+        <v>3</v>
+      </c>
+      <c r="X11" t="n">
+        <v>95</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>92</t>
         </is>
       </c>
     </row>
@@ -1480,9 +1550,15 @@
       <c r="V12" t="n">
         <v>3</v>
       </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>14</t>
+      <c r="W12" t="n">
+        <v>14</v>
+      </c>
+      <c r="X12" t="n">
+        <v>79</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>65</t>
         </is>
       </c>
     </row>
@@ -1571,9 +1647,15 @@
       <c r="V13" t="n">
         <v>3</v>
       </c>
-      <c r="W13" t="inlineStr">
-        <is>
-          <t>19</t>
+      <c r="W13" t="n">
+        <v>19</v>
+      </c>
+      <c r="X13" t="n">
+        <v>95</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>76</t>
         </is>
       </c>
     </row>
@@ -1656,9 +1738,15 @@
       <c r="V14" t="n">
         <v>51</v>
       </c>
-      <c r="W14" t="inlineStr">
-        <is>
-          <t>7</t>
+      <c r="W14" t="n">
+        <v>7</v>
+      </c>
+      <c r="X14" t="n">
+        <v>89</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>82</t>
         </is>
       </c>
     </row>
@@ -1743,9 +1831,15 @@
       <c r="V15" t="n">
         <v>3</v>
       </c>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>9</t>
+      <c r="W15" t="n">
+        <v>9</v>
+      </c>
+      <c r="X15" t="n">
+        <v>91</v>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>82</t>
         </is>
       </c>
     </row>
@@ -1834,9 +1928,15 @@
       <c r="V16" t="n">
         <v>4</v>
       </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>14</t>
+      <c r="W16" t="n">
+        <v>14</v>
+      </c>
+      <c r="X16" t="n">
+        <v>71</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>57</t>
         </is>
       </c>
     </row>
@@ -1884,6 +1984,8 @@
         <v>3</v>
       </c>
       <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1960,9 +2062,15 @@
       <c r="V18" t="n">
         <v>11</v>
       </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>4</t>
+      <c r="W18" t="n">
+        <v>4</v>
+      </c>
+      <c r="X18" t="n">
+        <v>87</v>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>83</t>
         </is>
       </c>
     </row>
@@ -2043,9 +2151,15 @@
       <c r="V19" t="n">
         <v>10</v>
       </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>30</t>
+      <c r="W19" t="n">
+        <v>30</v>
+      </c>
+      <c r="X19" t="n">
+        <v>99</v>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>69</t>
         </is>
       </c>
     </row>
@@ -2130,9 +2244,15 @@
       <c r="V20" t="n">
         <v>2</v>
       </c>
-      <c r="W20" t="inlineStr">
-        <is>
-          <t>17</t>
+      <c r="W20" t="n">
+        <v>17</v>
+      </c>
+      <c r="X20" t="n">
+        <v>75</v>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>58</t>
         </is>
       </c>
     </row>
@@ -2215,9 +2335,15 @@
       <c r="V21" t="n">
         <v>38</v>
       </c>
-      <c r="W21" t="inlineStr">
-        <is>
-          <t>18</t>
+      <c r="W21" t="n">
+        <v>18</v>
+      </c>
+      <c r="X21" t="n">
+        <v>75</v>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>57</t>
         </is>
       </c>
     </row>
@@ -2304,9 +2430,15 @@
       <c r="V22" t="n">
         <v>11</v>
       </c>
-      <c r="W22" t="inlineStr">
-        <is>
-          <t>12</t>
+      <c r="W22" t="n">
+        <v>12</v>
+      </c>
+      <c r="X22" t="n">
+        <v>105</v>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>93</t>
         </is>
       </c>
     </row>
@@ -2389,9 +2521,15 @@
       <c r="V23" t="n">
         <v>0</v>
       </c>
-      <c r="W23" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="W23" t="n">
+        <v>0</v>
+      </c>
+      <c r="X23" t="n">
+        <v>80</v>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>80</t>
         </is>
       </c>
     </row>
@@ -2478,9 +2616,15 @@
       <c r="V24" t="n">
         <v>4</v>
       </c>
-      <c r="W24" t="inlineStr">
-        <is>
-          <t>11</t>
+      <c r="W24" t="n">
+        <v>11</v>
+      </c>
+      <c r="X24" t="n">
+        <v>80</v>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>69</t>
         </is>
       </c>
     </row>
@@ -2567,9 +2711,15 @@
       <c r="V25" t="n">
         <v>2</v>
       </c>
-      <c r="W25" t="inlineStr">
-        <is>
-          <t>16</t>
+      <c r="W25" t="n">
+        <v>16</v>
+      </c>
+      <c r="X25" t="n">
+        <v>80</v>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>64</t>
         </is>
       </c>
     </row>
@@ -2659,6 +2809,8 @@
         <v>1</v>
       </c>
       <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2737,9 +2889,15 @@
       <c r="V27" t="n">
         <v>0</v>
       </c>
-      <c r="W27" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="W27" t="n">
+        <v>1</v>
+      </c>
+      <c r="X27" t="n">
+        <v>67</v>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>66</t>
         </is>
       </c>
     </row>
@@ -2829,6 +2987,8 @@
         <v>0</v>
       </c>
       <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2915,9 +3075,15 @@
       <c r="V29" t="n">
         <v>0</v>
       </c>
-      <c r="W29" t="inlineStr">
-        <is>
-          <t>11</t>
+      <c r="W29" t="n">
+        <v>11</v>
+      </c>
+      <c r="X29" t="n">
+        <v>80</v>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>69</t>
         </is>
       </c>
     </row>
@@ -3006,9 +3172,15 @@
       <c r="V30" t="n">
         <v>0</v>
       </c>
-      <c r="W30" t="inlineStr">
-        <is>
-          <t>4</t>
+      <c r="W30" t="n">
+        <v>4</v>
+      </c>
+      <c r="X30" t="n">
+        <v>67</v>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>63</t>
         </is>
       </c>
     </row>
@@ -3089,9 +3261,15 @@
       <c r="V31" t="n">
         <v>3</v>
       </c>
-      <c r="W31" t="inlineStr">
-        <is>
-          <t>7</t>
+      <c r="W31" t="n">
+        <v>7</v>
+      </c>
+      <c r="X31" t="n">
+        <v>74</v>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>67</t>
         </is>
       </c>
     </row>
@@ -3174,9 +3352,15 @@
       <c r="V32" t="n">
         <v>0</v>
       </c>
-      <c r="W32" t="inlineStr">
-        <is>
-          <t>9</t>
+      <c r="W32" t="n">
+        <v>9</v>
+      </c>
+      <c r="X32" t="n">
+        <v>90</v>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>81</t>
         </is>
       </c>
     </row>
@@ -3257,9 +3441,15 @@
       <c r="V33" t="n">
         <v>0</v>
       </c>
-      <c r="W33" t="inlineStr">
-        <is>
-          <t>4</t>
+      <c r="W33" t="n">
+        <v>4</v>
+      </c>
+      <c r="X33" t="n">
+        <v>64</v>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>60</t>
         </is>
       </c>
     </row>
@@ -3344,9 +3534,15 @@
       <c r="V34" t="n">
         <v>3</v>
       </c>
-      <c r="W34" t="inlineStr">
-        <is>
-          <t>7</t>
+      <c r="W34" t="n">
+        <v>7</v>
+      </c>
+      <c r="X34" t="n">
+        <v>75</v>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>68</t>
         </is>
       </c>
     </row>
@@ -3435,9 +3631,15 @@
       <c r="V35" t="n">
         <v>16</v>
       </c>
-      <c r="W35" t="inlineStr">
-        <is>
-          <t>25</t>
+      <c r="W35" t="n">
+        <v>25</v>
+      </c>
+      <c r="X35" t="n">
+        <v>96</v>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>71</t>
         </is>
       </c>
     </row>
@@ -3526,9 +3728,15 @@
       <c r="V36" t="n">
         <v>3</v>
       </c>
-      <c r="W36" t="inlineStr">
-        <is>
-          <t>12</t>
+      <c r="W36" t="n">
+        <v>12</v>
+      </c>
+      <c r="X36" t="n">
+        <v>81</v>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>69</t>
         </is>
       </c>
     </row>
@@ -3613,9 +3821,15 @@
       <c r="V37" t="n">
         <v>0</v>
       </c>
-      <c r="W37" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="W37" t="n">
+        <v>0</v>
+      </c>
+      <c r="X37" t="n">
+        <v>68</v>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>68</t>
         </is>
       </c>
     </row>
@@ -3704,9 +3918,15 @@
       <c r="V38" t="n">
         <v>6</v>
       </c>
-      <c r="W38" t="inlineStr">
-        <is>
-          <t>8</t>
+      <c r="W38" t="n">
+        <v>8</v>
+      </c>
+      <c r="X38" t="n">
+        <v>91</v>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>83</t>
         </is>
       </c>
     </row>
@@ -3791,9 +4011,15 @@
       <c r="V39" t="n">
         <v>11</v>
       </c>
-      <c r="W39" t="inlineStr">
-        <is>
-          <t>12</t>
+      <c r="W39" t="n">
+        <v>12</v>
+      </c>
+      <c r="X39" t="n">
+        <v>87</v>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>75</t>
         </is>
       </c>
     </row>
@@ -3880,9 +4106,15 @@
       <c r="V40" t="n">
         <v>7</v>
       </c>
-      <c r="W40" t="inlineStr">
-        <is>
-          <t>18</t>
+      <c r="W40" t="n">
+        <v>18</v>
+      </c>
+      <c r="X40" t="n">
+        <v>80</v>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>62</t>
         </is>
       </c>
     </row>
@@ -3971,9 +4203,15 @@
       <c r="V41" t="n">
         <v>0</v>
       </c>
-      <c r="W41" t="inlineStr">
-        <is>
-          <t>19</t>
+      <c r="W41" t="n">
+        <v>19</v>
+      </c>
+      <c r="X41" t="n">
+        <v>89</v>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>70</t>
         </is>
       </c>
     </row>
@@ -4050,9 +4288,15 @@
       <c r="V42" t="n">
         <v>1</v>
       </c>
-      <c r="W42" t="inlineStr">
-        <is>
-          <t>4</t>
+      <c r="W42" t="n">
+        <v>4</v>
+      </c>
+      <c r="X42" t="n">
+        <v>78</v>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>74</t>
         </is>
       </c>
     </row>
@@ -4141,9 +4385,15 @@
       <c r="V43" t="n">
         <v>4</v>
       </c>
-      <c r="W43" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="W43" t="n">
+        <v>1</v>
+      </c>
+      <c r="X43" t="n">
+        <v>84</v>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>83</t>
         </is>
       </c>
     </row>
@@ -4224,9 +4474,15 @@
       <c r="V44" t="n">
         <v>6</v>
       </c>
-      <c r="W44" t="inlineStr">
-        <is>
-          <t>8</t>
+      <c r="W44" t="n">
+        <v>8</v>
+      </c>
+      <c r="X44" t="n">
+        <v>78</v>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>70</t>
         </is>
       </c>
     </row>
@@ -4309,9 +4565,15 @@
       <c r="V45" t="n">
         <v>2</v>
       </c>
-      <c r="W45" t="inlineStr">
-        <is>
-          <t>19</t>
+      <c r="W45" t="n">
+        <v>19</v>
+      </c>
+      <c r="X45" t="n">
+        <v>88</v>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>69</t>
         </is>
       </c>
     </row>
@@ -4392,9 +4654,15 @@
       <c r="V46" t="n">
         <v>0</v>
       </c>
-      <c r="W46" t="inlineStr">
-        <is>
-          <t>6</t>
+      <c r="W46" t="n">
+        <v>6</v>
+      </c>
+      <c r="X46" t="n">
+        <v>77</v>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>71</t>
         </is>
       </c>
     </row>
@@ -4475,9 +4743,15 @@
       <c r="V47" t="n">
         <v>8</v>
       </c>
-      <c r="W47" t="inlineStr">
-        <is>
-          <t>24</t>
+      <c r="W47" t="n">
+        <v>24</v>
+      </c>
+      <c r="X47" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>61</t>
         </is>
       </c>
     </row>
@@ -4566,9 +4840,15 @@
       <c r="V48" t="n">
         <v>18</v>
       </c>
-      <c r="W48" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="W48" t="n">
+        <v>0</v>
+      </c>
+      <c r="X48" t="n">
+        <v>69</v>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>69</t>
         </is>
       </c>
     </row>
@@ -4653,9 +4933,15 @@
       <c r="V49" t="n">
         <v>0</v>
       </c>
-      <c r="W49" t="inlineStr">
-        <is>
-          <t>13</t>
+      <c r="W49" t="n">
+        <v>13</v>
+      </c>
+      <c r="X49" t="n">
+        <v>97</v>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>84</t>
         </is>
       </c>
     </row>
@@ -4738,9 +5024,15 @@
       <c r="V50" t="n">
         <v>8</v>
       </c>
-      <c r="W50" t="inlineStr">
-        <is>
-          <t>6</t>
+      <c r="W50" t="n">
+        <v>6</v>
+      </c>
+      <c r="X50" t="n">
+        <v>95</v>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>89</t>
         </is>
       </c>
     </row>
@@ -4827,9 +5119,15 @@
       <c r="V51" t="n">
         <v>12</v>
       </c>
-      <c r="W51" t="inlineStr">
-        <is>
-          <t>15</t>
+      <c r="W51" t="n">
+        <v>15</v>
+      </c>
+      <c r="X51" t="n">
+        <v>83</v>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>68</t>
         </is>
       </c>
     </row>
@@ -4910,9 +5208,15 @@
       <c r="V52" t="n">
         <v>0</v>
       </c>
-      <c r="W52" t="inlineStr">
-        <is>
-          <t>12</t>
+      <c r="W52" t="n">
+        <v>12</v>
+      </c>
+      <c r="X52" t="n">
+        <v>76</v>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>64</t>
         </is>
       </c>
     </row>
@@ -4993,9 +5297,15 @@
       <c r="V53" t="n">
         <v>6</v>
       </c>
-      <c r="W53" t="inlineStr">
-        <is>
-          <t>4</t>
+      <c r="W53" t="n">
+        <v>4</v>
+      </c>
+      <c r="X53" t="n">
+        <v>73</v>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>69</t>
         </is>
       </c>
     </row>
@@ -5049,6 +5359,8 @@
         <v>0</v>
       </c>
       <c r="W54" t="inlineStr"/>
+      <c r="X54" t="inlineStr"/>
+      <c r="Y54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5129,9 +5441,15 @@
         <v>2</v>
       </c>
       <c r="V55" t="inlineStr"/>
-      <c r="W55" t="inlineStr">
-        <is>
-          <t>26</t>
+      <c r="W55" t="n">
+        <v>26</v>
+      </c>
+      <c r="X55" t="n">
+        <v>90</v>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>64</t>
         </is>
       </c>
     </row>
@@ -5220,9 +5538,15 @@
       <c r="V56" t="n">
         <v>4</v>
       </c>
-      <c r="W56" t="inlineStr">
-        <is>
-          <t>20</t>
+      <c r="W56" t="n">
+        <v>20</v>
+      </c>
+      <c r="X56" t="n">
+        <v>89</v>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>69</t>
         </is>
       </c>
     </row>
@@ -5312,6 +5636,8 @@
         <v>3</v>
       </c>
       <c r="W57" t="inlineStr"/>
+      <c r="X57" t="inlineStr"/>
+      <c r="Y57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5390,9 +5716,15 @@
       <c r="V58" t="n">
         <v>1</v>
       </c>
-      <c r="W58" t="inlineStr">
-        <is>
-          <t>20</t>
+      <c r="W58" t="n">
+        <v>20</v>
+      </c>
+      <c r="X58" t="n">
+        <v>71</v>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>51</t>
         </is>
       </c>
     </row>
@@ -5482,6 +5814,8 @@
         <v>3</v>
       </c>
       <c r="W59" t="inlineStr"/>
+      <c r="X59" t="inlineStr"/>
+      <c r="Y59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5561,6 +5895,10 @@
         <v>1</v>
       </c>
       <c r="W60" t="inlineStr"/>
+      <c r="X60" t="n">
+        <v>87</v>
+      </c>
+      <c r="Y60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5647,9 +5985,15 @@
       <c r="V61" t="n">
         <v>3</v>
       </c>
-      <c r="W61" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="W61" t="n">
+        <v>0</v>
+      </c>
+      <c r="X61" t="n">
+        <v>61</v>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>61</t>
         </is>
       </c>
     </row>
@@ -5738,9 +6082,15 @@
       <c r="V62" t="n">
         <v>1</v>
       </c>
-      <c r="W62" t="inlineStr">
-        <is>
-          <t>20</t>
+      <c r="W62" t="n">
+        <v>20</v>
+      </c>
+      <c r="X62" t="n">
+        <v>66</v>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>46</t>
         </is>
       </c>
     </row>
@@ -5821,9 +6171,15 @@
       <c r="V63" t="n">
         <v>3</v>
       </c>
-      <c r="W63" t="inlineStr">
-        <is>
-          <t>5</t>
+      <c r="W63" t="n">
+        <v>5</v>
+      </c>
+      <c r="X63" t="n">
+        <v>79</v>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>74</t>
         </is>
       </c>
     </row>
@@ -5912,9 +6268,15 @@
       <c r="V64" t="n">
         <v>3</v>
       </c>
-      <c r="W64" t="inlineStr">
-        <is>
-          <t>18</t>
+      <c r="W64" t="n">
+        <v>18</v>
+      </c>
+      <c r="X64" t="n">
+        <v>86</v>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>68</t>
         </is>
       </c>
     </row>
@@ -5995,9 +6357,15 @@
       <c r="V65" t="n">
         <v>2</v>
       </c>
-      <c r="W65" t="inlineStr">
-        <is>
-          <t>10</t>
+      <c r="W65" t="n">
+        <v>10</v>
+      </c>
+      <c r="X65" t="n">
+        <v>72</v>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>62</t>
         </is>
       </c>
     </row>
@@ -6086,9 +6454,15 @@
       <c r="V66" t="n">
         <v>0</v>
       </c>
-      <c r="W66" t="inlineStr">
-        <is>
-          <t>34</t>
+      <c r="W66" t="n">
+        <v>34</v>
+      </c>
+      <c r="X66" t="n">
+        <v>69</v>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>35</t>
         </is>
       </c>
     </row>
@@ -6177,9 +6551,15 @@
       <c r="V67" t="n">
         <v>11</v>
       </c>
-      <c r="W67" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="W67" t="n">
+        <v>1</v>
+      </c>
+      <c r="X67" t="n">
+        <v>71</v>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>70</t>
         </is>
       </c>
     </row>
@@ -6256,9 +6636,15 @@
       <c r="V68" t="n">
         <v>9</v>
       </c>
-      <c r="W68" t="inlineStr">
-        <is>
-          <t>17</t>
+      <c r="W68" t="n">
+        <v>17</v>
+      </c>
+      <c r="X68" t="n">
+        <v>95</v>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>78</t>
         </is>
       </c>
     </row>
@@ -6345,9 +6731,15 @@
       <c r="V69" t="n">
         <v>3</v>
       </c>
-      <c r="W69" t="inlineStr">
-        <is>
-          <t>17</t>
+      <c r="W69" t="n">
+        <v>17</v>
+      </c>
+      <c r="X69" t="n">
+        <v>118</v>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>101</t>
         </is>
       </c>
     </row>
@@ -6436,9 +6828,15 @@
       <c r="V70" t="n">
         <v>0</v>
       </c>
-      <c r="W70" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="W70" t="n">
+        <v>0</v>
+      </c>
+      <c r="X70" t="n">
+        <v>70</v>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>70</t>
         </is>
       </c>
     </row>
@@ -6528,6 +6926,10 @@
         <v>3</v>
       </c>
       <c r="W71" t="inlineStr"/>
+      <c r="X71" t="n">
+        <v>78</v>
+      </c>
+      <c r="Y71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6614,9 +7016,15 @@
       <c r="V72" t="n">
         <v>10</v>
       </c>
-      <c r="W72" t="inlineStr">
-        <is>
-          <t>12</t>
+      <c r="W72" t="n">
+        <v>12</v>
+      </c>
+      <c r="X72" t="n">
+        <v>89</v>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>77</t>
         </is>
       </c>
     </row>
@@ -6705,9 +7113,15 @@
       <c r="V73" t="n">
         <v>4</v>
       </c>
-      <c r="W73" t="inlineStr">
-        <is>
-          <t>11</t>
+      <c r="W73" t="n">
+        <v>11</v>
+      </c>
+      <c r="X73" t="n">
+        <v>79</v>
+      </c>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>68</t>
         </is>
       </c>
     </row>
@@ -6788,9 +7202,15 @@
       <c r="V74" t="n">
         <v>3</v>
       </c>
-      <c r="W74" t="inlineStr">
-        <is>
-          <t>6</t>
+      <c r="W74" t="n">
+        <v>6</v>
+      </c>
+      <c r="X74" t="n">
+        <v>80</v>
+      </c>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>74</t>
         </is>
       </c>
     </row>
@@ -6879,9 +7299,15 @@
       <c r="V75" t="n">
         <v>2</v>
       </c>
-      <c r="W75" t="inlineStr">
-        <is>
-          <t>24</t>
+      <c r="W75" t="n">
+        <v>24</v>
+      </c>
+      <c r="X75" t="n">
+        <v>69</v>
+      </c>
+      <c r="Y75" t="inlineStr">
+        <is>
+          <t>45</t>
         </is>
       </c>
     </row>
@@ -6966,9 +7392,15 @@
       <c r="V76" t="n">
         <v>17</v>
       </c>
-      <c r="W76" t="inlineStr">
-        <is>
-          <t>18</t>
+      <c r="W76" t="n">
+        <v>18</v>
+      </c>
+      <c r="X76" t="n">
+        <v>81</v>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>63</t>
         </is>
       </c>
     </row>
@@ -7049,9 +7481,15 @@
       <c r="V77" t="n">
         <v>24</v>
       </c>
-      <c r="W77" t="inlineStr">
-        <is>
-          <t>16</t>
+      <c r="W77" t="n">
+        <v>16</v>
+      </c>
+      <c r="X77" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>69</t>
         </is>
       </c>
     </row>
@@ -7129,6 +7567,8 @@
         <v>3</v>
       </c>
       <c r="W78" t="inlineStr"/>
+      <c r="X78" t="inlineStr"/>
+      <c r="Y78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7208,6 +7648,8 @@
         <v>0</v>
       </c>
       <c r="W79" t="inlineStr"/>
+      <c r="X79" t="inlineStr"/>
+      <c r="Y79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -7294,9 +7736,15 @@
       <c r="V80" t="n">
         <v>2</v>
       </c>
-      <c r="W80" t="inlineStr">
-        <is>
-          <t>8</t>
+      <c r="W80" t="n">
+        <v>8</v>
+      </c>
+      <c r="X80" t="n">
+        <v>91</v>
+      </c>
+      <c r="Y80" t="inlineStr">
+        <is>
+          <t>83</t>
         </is>
       </c>
     </row>
@@ -7380,6 +7828,8 @@
         <v>2</v>
       </c>
       <c r="W81" t="inlineStr"/>
+      <c r="X81" t="inlineStr"/>
+      <c r="Y81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7458,9 +7908,15 @@
       <c r="V82" t="n">
         <v>2</v>
       </c>
-      <c r="W82" t="inlineStr">
-        <is>
-          <t>10</t>
+      <c r="W82" t="n">
+        <v>10</v>
+      </c>
+      <c r="X82" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y82" t="inlineStr">
+        <is>
+          <t>48</t>
         </is>
       </c>
     </row>
@@ -7549,9 +8005,15 @@
       <c r="V83" t="n">
         <v>29</v>
       </c>
-      <c r="W83" t="inlineStr">
-        <is>
-          <t>16</t>
+      <c r="W83" t="n">
+        <v>16</v>
+      </c>
+      <c r="X83" t="n">
+        <v>88</v>
+      </c>
+      <c r="Y83" t="inlineStr">
+        <is>
+          <t>72</t>
         </is>
       </c>
     </row>
@@ -7639,6 +8101,8 @@
         <v>10</v>
       </c>
       <c r="W84" t="inlineStr"/>
+      <c r="X84" t="inlineStr"/>
+      <c r="Y84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7720,6 +8184,10 @@
         <v>0</v>
       </c>
       <c r="W85" t="inlineStr"/>
+      <c r="X85" t="n">
+        <v>60</v>
+      </c>
+      <c r="Y85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7800,9 +8268,15 @@
       <c r="V86" t="n">
         <v>5</v>
       </c>
-      <c r="W86" t="inlineStr">
-        <is>
-          <t>9</t>
+      <c r="W86" t="n">
+        <v>9</v>
+      </c>
+      <c r="X86" t="n">
+        <v>94</v>
+      </c>
+      <c r="Y86" t="inlineStr">
+        <is>
+          <t>85</t>
         </is>
       </c>
     </row>

</xml_diff>